<commit_message>
Add  required pdf documents
</commit_message>
<xml_diff>
--- a/Test_Cases_saucedemo.xlsx
+++ b/Test_Cases_saucedemo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\Technical Assessment - Automation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5DD61E96-BFCB-404E-B76A-8B30D63EED4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FAE9F2D4-7F1B-4F01-A446-226500121035}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{577270D6-3CE9-469C-A4A8-B56522A6439E}"/>
+    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{577270D6-3CE9-469C-A4A8-B56522A6439E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="110">
   <si>
     <t>Test Case ID </t>
   </si>
@@ -72,10 +72,6 @@
   </si>
   <si>
     <t>Modules Covered :</t>
-  </si>
-  <si>
-    <t>Login, Product Browsing 
-Cart, Checkout</t>
   </si>
   <si>
     <t>TC_01</t>
@@ -162,10 +158,6 @@
 03. Click the login button.</t>
   </si>
   <si>
-    <t>System display an error 
-message and block access</t>
-  </si>
-  <si>
     <t>Check the login functionality with 
 empty username and password</t>
   </si>
@@ -201,10 +193,6 @@
   <si>
     <t>01.Click filter drop down menu
 02.Select Price(High to low)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Check Item sorting  feature with
-Price(High to low) option</t>
   </si>
   <si>
     <t xml:space="preserve">Logged in as problem_user.
@@ -212,10 +200,6 @@
 </t>
   </si>
   <si>
-    <t>01.Select a added item in the inventory
-02.Click  "Remove" buttons item</t>
-  </si>
-  <si>
     <t>Item should be 
 removed from the cart."Remove" button change to "Add to cart"</t>
   </si>
@@ -257,12 +241,6 @@
  form validation</t>
   </si>
   <si>
-    <t xml:space="preserve">
-01.Enter valid First Name
-02.Enter valid Last Name
-03.Enter letter in  Zip/Postal code field</t>
-  </si>
-  <si>
     <t>First Name : Syura
 Last Name : Chalana
 Zip/Postal code : Postal1</t>
@@ -293,16 +271,8 @@
 </t>
   </si>
   <si>
-    <t>System display 
-all added items ,Payment Information,
-Shipping Information,Price Total</t>
-  </si>
-  <si>
     <t>Validate Checkout: 
 Overview information ui</t>
-  </si>
-  <si>
-    <t>Check Your information Form behavivour</t>
   </si>
   <si>
     <t>System calculates total price correctly</t>
@@ -329,10 +299,6 @@
     <t>System should redirect the user to the Checkout page.</t>
   </si>
   <si>
-    <t xml:space="preserve">01.Click cart icon on inventory ui
-02.Click  "Checkout" buttons </t>
-  </si>
-  <si>
     <t>System displays "Error: First Name is required" message.</t>
   </si>
   <si>
@@ -363,11 +329,6 @@
     <t>System displays abnormal behavior when entering text in the Last Name field. 
 While typing in the Last Name field, the  First Name field updates, 
 with characters appearing one at a time.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">
-01.Keep all fields empty
-02.Click  "Checkout" buttons </t>
   </si>
   <si>
     <t xml:space="preserve">
@@ -401,20 +362,8 @@
 Total: $64.78</t>
   </si>
   <si>
-    <t>System should calculate total price 
-correctly  with tax. And should rounded to two decimal places.</t>
-  </si>
-  <si>
     <t>Drop down menu select specified option.All items sorted on prices, 
 from high to low</t>
-  </si>
-  <si>
-    <t>System sorted items according to prices, 
-from from high to low</t>
-  </si>
-  <si>
-    <t>1. Select an items from the inventory list/ui.
-2. Click the "Add to Cart" button for all items.</t>
   </si>
   <si>
     <t>Items are added to the 
@@ -437,10 +386,63 @@
 </t>
   </si>
   <si>
-    <t>Validate final total calculation for problem_user</t>
-  </si>
-  <si>
     <t>Validate final total calculation for standard_user</t>
+  </si>
+  <si>
+    <t>Validate final total calculation for  visual_user</t>
+  </si>
+  <si>
+    <t>Verify Price (High to Low) sort filter fails for problem_user</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verify Price (High to Low) sort filter fails for  standard_user </t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+01.Keep all fields empty
+02.Click  "Continue" buttons </t>
+  </si>
+  <si>
+    <t>Check Your information Form behaviour</t>
+  </si>
+  <si>
+    <t>01. Select an items from the inventory list/ui.
+02. Click the "Add to Cart" button for all items.</t>
+  </si>
+  <si>
+    <t>Login, Product Browsing, 
+Cart, Checkout</t>
+  </si>
+  <si>
+    <t>System displays an error 
+message and block access</t>
+  </si>
+  <si>
+    <t>System sorted items according to prices, 
+from high to low</t>
+  </si>
+  <si>
+    <t xml:space="preserve">01.Click cart icon on inventory ui
+02.Click  "Checkout" button </t>
+  </si>
+  <si>
+    <t>01.Select an added item in the inventory
+02.Click  "Remove" button item</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+01.Enter valid First Name
+02.Enter valid Last Name
+03.Enter valid  Zip/Postal code field</t>
+  </si>
+  <si>
+    <t>System displays
+all added items ,Payment Information,
+Shipping Information,Price Total</t>
+  </si>
+  <si>
+    <t>System should calculate total price 
+correctly  with tax. And should be rounded to two decimal places.</t>
   </si>
 </sst>
 </file>
@@ -998,7 +1000,7 @@
         <v>10</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>11</v>
+        <v>102</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
@@ -1012,16 +1014,16 @@
         <v>1</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="E7" s="2" t="s">
         <v>2</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="G7" s="2" t="s">
         <v>3</v>
@@ -1035,446 +1037,446 @@
     </row>
     <row r="8" spans="1:10" ht="77.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B8" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="C8" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="D8" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="E8" s="13" t="s">
         <v>31</v>
       </c>
-      <c r="C8" s="8" t="s">
+      <c r="F8" s="13" t="s">
+        <v>39</v>
+      </c>
+      <c r="G8" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="H8" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="I8" s="15" t="s">
         <v>33</v>
-      </c>
-      <c r="D8" s="8" t="s">
-        <v>45</v>
-      </c>
-      <c r="E8" s="13" t="s">
-        <v>32</v>
-      </c>
-      <c r="F8" s="13" t="s">
-        <v>41</v>
-      </c>
-      <c r="G8" s="8" t="s">
-        <v>55</v>
-      </c>
-      <c r="H8" s="8" t="s">
-        <v>55</v>
-      </c>
-      <c r="I8" s="15" t="s">
-        <v>34</v>
       </c>
     </row>
     <row r="9" spans="1:10" ht="77.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="9" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C9" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="D9" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="E9" s="13" t="s">
         <v>35</v>
       </c>
-      <c r="D9" s="8" t="s">
-        <v>45</v>
-      </c>
-      <c r="E9" s="13" t="s">
-        <v>36</v>
-      </c>
       <c r="F9" s="13" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="H9" s="8" t="s">
-        <v>37</v>
+        <v>103</v>
       </c>
       <c r="I9" s="15" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="10" spans="1:10" ht="77.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="9" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C10" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="D10" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="E10" s="13" t="s">
+        <v>37</v>
+      </c>
+      <c r="F10" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="G10" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="D10" s="8" t="s">
-        <v>45</v>
-      </c>
-      <c r="E10" s="13" t="s">
-        <v>39</v>
-      </c>
-      <c r="F10" s="13" t="s">
-        <v>43</v>
-      </c>
-      <c r="G10" s="8" t="s">
-        <v>40</v>
-      </c>
       <c r="H10" s="8" t="s">
-        <v>86</v>
+        <v>78</v>
       </c>
       <c r="I10" s="15" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="11" spans="1:10" ht="77.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>75</v>
+        <v>68</v>
       </c>
       <c r="E11" s="13" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="F11" s="8" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="H11" s="8" t="s">
-        <v>87</v>
+        <v>79</v>
       </c>
       <c r="I11" s="15" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="12" spans="1:10" ht="77.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="9" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>48</v>
+        <v>98</v>
       </c>
       <c r="D12" s="8" t="s">
-        <v>75</v>
+        <v>68</v>
       </c>
       <c r="E12" s="13" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="F12" s="8" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="G12" s="8" t="s">
-        <v>99</v>
+        <v>89</v>
       </c>
       <c r="H12" s="8" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="I12" s="15" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="13" spans="1:10" ht="77.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="9" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>48</v>
+        <v>97</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>76</v>
+        <v>69</v>
       </c>
       <c r="E13" s="13" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="F13" s="8" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="G13" s="8" t="s">
-        <v>93</v>
+        <v>84</v>
       </c>
       <c r="H13" s="8" t="s">
-        <v>92</v>
+        <v>83</v>
       </c>
       <c r="I13" s="16" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="14" spans="1:10" ht="77.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="9" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C14" s="11" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>77</v>
+        <v>70</v>
       </c>
       <c r="E14" s="13" t="s">
-        <v>78</v>
+        <v>71</v>
       </c>
       <c r="F14" s="8" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="G14" s="8" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="H14" s="8" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="I14" s="15" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="15" spans="1:10" ht="77.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="9" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C15" s="11" t="s">
-        <v>83</v>
+        <v>75</v>
       </c>
       <c r="D15" s="8" t="s">
-        <v>76</v>
+        <v>69</v>
       </c>
       <c r="E15" s="13" t="s">
         <v>101</v>
       </c>
       <c r="F15" s="8" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="G15" s="8" t="s">
-        <v>102</v>
+        <v>90</v>
       </c>
       <c r="H15" s="8" t="s">
-        <v>103</v>
+        <v>91</v>
       </c>
       <c r="I15" s="17" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="J15" s="18"/>
     </row>
     <row r="16" spans="1:10" ht="77.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="9" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B16" s="11" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>105</v>
+        <v>93</v>
       </c>
       <c r="D16" s="8" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="E16" s="13" t="s">
-        <v>50</v>
+        <v>106</v>
       </c>
       <c r="F16" s="8" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="G16" s="8" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="H16" s="8" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="I16" s="17" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="J16" s="18"/>
     </row>
     <row r="17" spans="1:11" ht="77.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="9" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B17" s="11" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C17" s="11" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="D17" s="8" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="E17" s="13" t="s">
-        <v>80</v>
+        <v>105</v>
       </c>
       <c r="F17" s="8" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="G17" s="8" t="s">
-        <v>79</v>
+        <v>72</v>
       </c>
       <c r="H17" s="11" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="I17" s="15" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="18" spans="1:11" ht="120" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="9" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>72</v>
+        <v>100</v>
       </c>
       <c r="D18" s="8" t="s">
-        <v>85</v>
+        <v>77</v>
       </c>
       <c r="E18" s="13" t="s">
-        <v>62</v>
+        <v>107</v>
       </c>
       <c r="F18" s="8" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="G18" s="8" t="s">
-        <v>84</v>
+        <v>76</v>
       </c>
       <c r="H18" s="8" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="I18" s="17" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="J18" s="14"/>
     </row>
     <row r="19" spans="1:11" ht="77.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="9" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B19" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="C19" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="D19" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="E19" s="13" t="s">
+        <v>99</v>
+      </c>
+      <c r="F19" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="G19" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="C19" s="8" t="s">
-        <v>64</v>
-      </c>
-      <c r="D19" s="8" t="s">
-        <v>68</v>
-      </c>
-      <c r="E19" s="13" t="s">
-        <v>90</v>
-      </c>
-      <c r="F19" s="12" t="s">
-        <v>65</v>
-      </c>
-      <c r="G19" s="8" t="s">
-        <v>66</v>
-      </c>
       <c r="H19" s="8" t="s">
-        <v>81</v>
+        <v>73</v>
       </c>
       <c r="I19" s="15" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="20" spans="1:11" ht="77.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="9" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B20" s="11" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C20" s="8" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="D20" s="8" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="E20" s="13" t="s">
-        <v>91</v>
+        <v>82</v>
       </c>
       <c r="F20" s="8" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="G20" s="8" t="s">
-        <v>70</v>
+        <v>108</v>
       </c>
       <c r="H20" s="8" t="s">
-        <v>74</v>
+        <v>67</v>
       </c>
       <c r="I20" s="15" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="21" spans="1:11" ht="77.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="9" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B21" s="11" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C21" s="8" t="s">
-        <v>107</v>
+        <v>95</v>
       </c>
       <c r="D21" s="8" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="E21" s="13" t="s">
-        <v>95</v>
+        <v>86</v>
       </c>
       <c r="F21" s="8" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="G21" s="8" t="s">
-        <v>82</v>
+        <v>74</v>
       </c>
       <c r="H21" s="8" t="s">
-        <v>73</v>
+        <v>66</v>
       </c>
       <c r="I21" s="15" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="22" spans="1:11" ht="91.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="B22" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="C22" s="8" t="s">
+        <v>96</v>
+      </c>
+      <c r="D22" s="8" t="s">
         <v>94</v>
       </c>
-      <c r="B22" s="11" t="s">
-        <v>28</v>
-      </c>
-      <c r="C22" s="8" t="s">
-        <v>108</v>
-      </c>
-      <c r="D22" s="8" t="s">
-        <v>106</v>
-      </c>
       <c r="E22" s="13" t="s">
-        <v>95</v>
+        <v>86</v>
       </c>
       <c r="F22" s="8" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="G22" s="8" t="s">
-        <v>98</v>
+        <v>109</v>
       </c>
       <c r="H22" s="8" t="s">
-        <v>97</v>
+        <v>88</v>
       </c>
       <c r="I22" s="17" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="J22" t="s">
-        <v>96</v>
+        <v>87</v>
       </c>
       <c r="K22" s="18" t="s">
-        <v>104</v>
+        <v>92</v>
       </c>
     </row>
     <row r="23" spans="1:11" ht="66.75" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>